<commit_message>
Add template formatting, account structure step, and row hiding
- All 3 templates now have shading: cream fill for data entry zones,
  gray fill for totals, orange bold for section headers, thin borders
- New Step 3 "Account Structure" in generator: BS accounts (assets,
  liabilities, equity) and P&L accounts (revenue, COGS, expenses,
  other income/expense)
- Excess blank rows hidden based on account counts using SheetJS !rows
- Generator is now 5 steps: Type → Complexity → Accounts → Details → Review

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/1065_WTB_Template.xlsx
+++ b/templates/1065_WTB_Template.xlsx
@@ -27,7 +27,7 @@
     <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
     <numFmt numFmtId="165" formatCode="\+#,##0;\-#,##0;0"/>
   </numFmts>
-  <fonts count="38">
+  <fonts count="42">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -296,8 +296,31 @@
       <i val="1"/>
       <color rgb="00999999"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00F07840"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00F07840"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -375,8 +398,20 @@
         <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF8E7"/>
+        <bgColor rgb="00FFF8E7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F0F0"/>
+        <bgColor rgb="00F0F0F0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="8">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -433,6 +468,25 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D0D0D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D0D0"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="00808080"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -444,7 +498,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="209">
+  <cellXfs count="231">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1065,6 +1119,70 @@
     </xf>
     <xf numFmtId="0" fontId="37" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="36" fillId="14" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="15" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="32" fillId="15" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="32" fillId="15" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="22" fillId="15" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="15" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="15" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1328,19 +1446,20 @@
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="104">
-      <c r="A1" s="105" t="inlineStr">
+      <c r="A1" s="209" t="inlineStr">
         <is>
           <t>[ENTITY NAME]</t>
         </is>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="104">
-      <c r="A2" s="106" t="inlineStr">
+      <c r="A2" s="210" t="inlineStr">
         <is>
           <t>EIN: [XX-XXXXXXX]  |  Tax Year: [Start] - [End]  |  [Accrual/Cash] Basis  |  [#] Partners ([Split])</t>
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="104">
       <c r="A4" s="107" t="inlineStr">
         <is>
@@ -1364,7 +1483,7 @@
       </c>
     </row>
     <row r="5" ht="21.75" customHeight="1" s="104">
-      <c r="A5" s="108" t="inlineStr">
+      <c r="A5" s="211" t="inlineStr">
         <is>
           <t>ASSETS</t>
         </is>
@@ -1384,8 +1503,8 @@
           <t>Cash - Operating</t>
         </is>
       </c>
-      <c r="C6" s="111" t="n"/>
-      <c r="D6" s="112" t="n"/>
+      <c r="C6" s="212" t="n"/>
+      <c r="D6" s="213" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1" s="104">
       <c r="A7" s="109" t="inlineStr">
@@ -1398,8 +1517,8 @@
           <t>Cash - Savings</t>
         </is>
       </c>
-      <c r="C7" s="111" t="n"/>
-      <c r="D7" s="112" t="n"/>
+      <c r="C7" s="212" t="n"/>
+      <c r="D7" s="213" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1" s="104">
       <c r="A8" s="109" t="inlineStr">
@@ -1412,8 +1531,8 @@
           <t>Petty Cash</t>
         </is>
       </c>
-      <c r="C8" s="111" t="n"/>
-      <c r="D8" s="112" t="n"/>
+      <c r="C8" s="212" t="n"/>
+      <c r="D8" s="213" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1" s="104">
       <c r="A9" s="109" t="inlineStr">
@@ -1426,8 +1545,8 @@
           <t>Accounts Receivable</t>
         </is>
       </c>
-      <c r="C9" s="111" t="n"/>
-      <c r="D9" s="112" t="n"/>
+      <c r="C9" s="212" t="n"/>
+      <c r="D9" s="213" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="104">
       <c r="A10" s="109" t="inlineStr">
@@ -1440,8 +1559,8 @@
           <t>Allowance for Doubtful Accounts</t>
         </is>
       </c>
-      <c r="C10" s="112" t="n"/>
-      <c r="D10" s="111" t="n"/>
+      <c r="C10" s="213" t="n"/>
+      <c r="D10" s="212" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="104">
       <c r="A11" s="109" t="inlineStr">
@@ -1454,8 +1573,8 @@
           <t>Notes Receivable - Current</t>
         </is>
       </c>
-      <c r="C11" s="111" t="n"/>
-      <c r="D11" s="112" t="n"/>
+      <c r="C11" s="212" t="n"/>
+      <c r="D11" s="213" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1" s="104">
       <c r="A12" s="113" t="inlineStr">
@@ -1468,8 +1587,8 @@
           <t>Inventory (MUST = PY Ending Inventory)</t>
         </is>
       </c>
-      <c r="C12" s="111" t="n"/>
-      <c r="D12" s="112" t="n"/>
+      <c r="C12" s="212" t="n"/>
+      <c r="D12" s="213" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1" s="104">
       <c r="A13" s="109" t="inlineStr">
@@ -1482,8 +1601,8 @@
           <t>Prepaid Insurance</t>
         </is>
       </c>
-      <c r="C13" s="111" t="n"/>
-      <c r="D13" s="112" t="n"/>
+      <c r="C13" s="212" t="n"/>
+      <c r="D13" s="213" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="104">
       <c r="A14" s="109" t="inlineStr">
@@ -1496,8 +1615,8 @@
           <t>Prepaid Rent</t>
         </is>
       </c>
-      <c r="C14" s="111" t="n"/>
-      <c r="D14" s="112" t="n"/>
+      <c r="C14" s="212" t="n"/>
+      <c r="D14" s="213" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="104">
       <c r="A15" s="109" t="inlineStr">
@@ -1510,8 +1629,8 @@
           <t>Investments - Stocks (Short-term)</t>
         </is>
       </c>
-      <c r="C15" s="111" t="n"/>
-      <c r="D15" s="112" t="n"/>
+      <c r="C15" s="212" t="n"/>
+      <c r="D15" s="213" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="104">
       <c r="A16" s="109" t="inlineStr">
@@ -1524,8 +1643,8 @@
           <t>Investments - Municipal Bonds</t>
         </is>
       </c>
-      <c r="C16" s="111" t="n"/>
-      <c r="D16" s="112" t="n"/>
+      <c r="C16" s="212" t="n"/>
+      <c r="D16" s="213" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="104">
       <c r="A17" s="109" t="inlineStr">
@@ -1538,8 +1657,8 @@
           <t>Investments - Corporate Bonds</t>
         </is>
       </c>
-      <c r="C17" s="111" t="n"/>
-      <c r="D17" s="112" t="n"/>
+      <c r="C17" s="212" t="n"/>
+      <c r="D17" s="213" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="104">
       <c r="A18" s="109" t="inlineStr">
@@ -1552,8 +1671,8 @@
           <t>Loans to Partners</t>
         </is>
       </c>
-      <c r="C18" s="111" t="n"/>
-      <c r="D18" s="112" t="n"/>
+      <c r="C18" s="212" t="n"/>
+      <c r="D18" s="213" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1" s="104">
       <c r="A19" s="109" t="inlineStr">
@@ -1566,8 +1685,8 @@
           <t>Land</t>
         </is>
       </c>
-      <c r="C19" s="111" t="n"/>
-      <c r="D19" s="112" t="n"/>
+      <c r="C19" s="212" t="n"/>
+      <c r="D19" s="213" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1" s="104">
       <c r="A20" s="109" t="inlineStr">
@@ -1580,8 +1699,8 @@
           <t>Buildings</t>
         </is>
       </c>
-      <c r="C20" s="111" t="n"/>
-      <c r="D20" s="112" t="n"/>
+      <c r="C20" s="212" t="n"/>
+      <c r="D20" s="213" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="104">
       <c r="A21" s="109" t="inlineStr">
@@ -1594,8 +1713,8 @@
           <t>Accum Depreciation - Buildings</t>
         </is>
       </c>
-      <c r="C21" s="112" t="n"/>
-      <c r="D21" s="111" t="n"/>
+      <c r="C21" s="213" t="n"/>
+      <c r="D21" s="212" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="104">
       <c r="A22" s="109" t="inlineStr">
@@ -1608,8 +1727,8 @@
           <t>Furniture &amp; Fixtures</t>
         </is>
       </c>
-      <c r="C22" s="111" t="n"/>
-      <c r="D22" s="112" t="n"/>
+      <c r="C22" s="212" t="n"/>
+      <c r="D22" s="213" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1" s="104">
       <c r="A23" s="109" t="inlineStr">
@@ -1622,8 +1741,8 @@
           <t>Accum Depreciation - Furn &amp; Fix</t>
         </is>
       </c>
-      <c r="C23" s="112" t="n"/>
-      <c r="D23" s="111" t="n"/>
+      <c r="C23" s="213" t="n"/>
+      <c r="D23" s="212" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1" s="104">
       <c r="A24" s="109" t="inlineStr">
@@ -1636,8 +1755,8 @@
           <t>Vehicles</t>
         </is>
       </c>
-      <c r="C24" s="111" t="n"/>
-      <c r="D24" s="112" t="n"/>
+      <c r="C24" s="212" t="n"/>
+      <c r="D24" s="213" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1" s="104">
       <c r="A25" s="109" t="inlineStr">
@@ -1650,8 +1769,8 @@
           <t>Accum Depreciation - Vehicles</t>
         </is>
       </c>
-      <c r="C25" s="112" t="n"/>
-      <c r="D25" s="111" t="n"/>
+      <c r="C25" s="213" t="n"/>
+      <c r="D25" s="212" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1" s="104">
       <c r="A26" s="109" t="inlineStr">
@@ -1664,8 +1783,8 @@
           <t>Equipment</t>
         </is>
       </c>
-      <c r="C26" s="111" t="n"/>
-      <c r="D26" s="112" t="n"/>
+      <c r="C26" s="212" t="n"/>
+      <c r="D26" s="213" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="104">
       <c r="A27" s="109" t="inlineStr">
@@ -1678,8 +1797,8 @@
           <t>Accum Depreciation - Equipment</t>
         </is>
       </c>
-      <c r="C27" s="112" t="n"/>
-      <c r="D27" s="111" t="n"/>
+      <c r="C27" s="213" t="n"/>
+      <c r="D27" s="212" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1" s="104">
       <c r="A28" s="109" t="inlineStr">
@@ -1692,8 +1811,8 @@
           <t>Leasehold Improvements</t>
         </is>
       </c>
-      <c r="C28" s="111" t="n"/>
-      <c r="D28" s="112" t="n"/>
+      <c r="C28" s="212" t="n"/>
+      <c r="D28" s="213" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1" s="104">
       <c r="A29" s="109" t="inlineStr">
@@ -1706,8 +1825,8 @@
           <t>Accum Amort - Leasehold Impr</t>
         </is>
       </c>
-      <c r="C29" s="112" t="n"/>
-      <c r="D29" s="111" t="n"/>
+      <c r="C29" s="213" t="n"/>
+      <c r="D29" s="212" t="n"/>
     </row>
     <row r="30" ht="15" customHeight="1" s="104">
       <c r="A30" s="109" t="inlineStr">
@@ -1720,8 +1839,8 @@
           <t>Goodwill (Acquired)</t>
         </is>
       </c>
-      <c r="C30" s="111" t="n"/>
-      <c r="D30" s="112" t="n"/>
+      <c r="C30" s="212" t="n"/>
+      <c r="D30" s="213" t="n"/>
     </row>
     <row r="31" ht="15" customHeight="1" s="104">
       <c r="A31" s="109" t="inlineStr">
@@ -1734,8 +1853,8 @@
           <t>Accum Amort - Goodwill</t>
         </is>
       </c>
-      <c r="C31" s="112" t="n"/>
-      <c r="D31" s="111" t="n"/>
+      <c r="C31" s="213" t="n"/>
+      <c r="D31" s="212" t="n"/>
     </row>
     <row r="32" ht="15" customHeight="1" s="104">
       <c r="A32" s="109" t="inlineStr">
@@ -1748,8 +1867,8 @@
           <t>Patents</t>
         </is>
       </c>
-      <c r="C32" s="111" t="n"/>
-      <c r="D32" s="112" t="n"/>
+      <c r="C32" s="212" t="n"/>
+      <c r="D32" s="213" t="n"/>
     </row>
     <row r="33" ht="15" customHeight="1" s="104">
       <c r="A33" s="109" t="inlineStr">
@@ -1762,8 +1881,8 @@
           <t>Accum Amort - Patents</t>
         </is>
       </c>
-      <c r="C33" s="112" t="n"/>
-      <c r="D33" s="111" t="n"/>
+      <c r="C33" s="213" t="n"/>
+      <c r="D33" s="212" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1" s="104">
       <c r="A34" s="109" t="inlineStr">
@@ -1776,8 +1895,8 @@
           <t>Security Deposits</t>
         </is>
       </c>
-      <c r="C34" s="111" t="n"/>
-      <c r="D34" s="112" t="n"/>
+      <c r="C34" s="212" t="n"/>
+      <c r="D34" s="213" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1" s="104">
       <c r="A35" s="109" t="inlineStr">
@@ -1790,11 +1909,11 @@
           <t>Investment in Sub-Partnership (K-1 received)</t>
         </is>
       </c>
-      <c r="C35" s="111" t="n"/>
-      <c r="D35" s="112" t="n"/>
+      <c r="C35" s="212" t="n"/>
+      <c r="D35" s="213" t="n"/>
     </row>
     <row r="36" ht="21.75" customHeight="1" s="104">
-      <c r="A36" s="108" t="inlineStr">
+      <c r="A36" s="211" t="inlineStr">
         <is>
           <t>LIABILITIES</t>
         </is>
@@ -1814,8 +1933,8 @@
           <t>Accounts Payable</t>
         </is>
       </c>
-      <c r="C37" s="112" t="n"/>
-      <c r="D37" s="111" t="n"/>
+      <c r="C37" s="213" t="n"/>
+      <c r="D37" s="212" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1" s="104">
       <c r="A38" s="109" t="inlineStr">
@@ -1828,8 +1947,8 @@
           <t>Accrued Expenses</t>
         </is>
       </c>
-      <c r="C38" s="112" t="n"/>
-      <c r="D38" s="111" t="n"/>
+      <c r="C38" s="213" t="n"/>
+      <c r="D38" s="212" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1" s="104">
       <c r="A39" s="109" t="inlineStr">
@@ -1842,8 +1961,8 @@
           <t>Accrued Payroll &amp; Payroll Taxes</t>
         </is>
       </c>
-      <c r="C39" s="112" t="n"/>
-      <c r="D39" s="111" t="n"/>
+      <c r="C39" s="213" t="n"/>
+      <c r="D39" s="212" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1" s="104">
       <c r="A40" s="109" t="inlineStr">
@@ -1856,8 +1975,8 @@
           <t>Accrued Bonuses - Related Party (&gt;2.5 mo unpaid)</t>
         </is>
       </c>
-      <c r="C40" s="112" t="n"/>
-      <c r="D40" s="111" t="n"/>
+      <c r="C40" s="213" t="n"/>
+      <c r="D40" s="212" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1" s="104">
       <c r="A41" s="109" t="inlineStr">
@@ -1870,8 +1989,8 @@
           <t>Sales Tax Payable</t>
         </is>
       </c>
-      <c r="C41" s="112" t="n"/>
-      <c r="D41" s="111" t="n"/>
+      <c r="C41" s="213" t="n"/>
+      <c r="D41" s="212" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1" s="104">
       <c r="A42" s="109" t="inlineStr">
@@ -1884,8 +2003,8 @@
           <t>Unearned Revenue / Deferred Revenue</t>
         </is>
       </c>
-      <c r="C42" s="112" t="n"/>
-      <c r="D42" s="111" t="n"/>
+      <c r="C42" s="213" t="n"/>
+      <c r="D42" s="212" t="n"/>
     </row>
     <row r="43" ht="15" customHeight="1" s="104">
       <c r="A43" s="109" t="inlineStr">
@@ -1898,8 +2017,8 @@
           <t>Line of Credit</t>
         </is>
       </c>
-      <c r="C43" s="112" t="n"/>
-      <c r="D43" s="111" t="n"/>
+      <c r="C43" s="213" t="n"/>
+      <c r="D43" s="212" t="n"/>
     </row>
     <row r="44" ht="15" customHeight="1" s="104">
       <c r="A44" s="109" t="inlineStr">
@@ -1912,8 +2031,8 @@
           <t>Note Payable - Bank (Current Portion)</t>
         </is>
       </c>
-      <c r="C44" s="112" t="n"/>
-      <c r="D44" s="111" t="n"/>
+      <c r="C44" s="213" t="n"/>
+      <c r="D44" s="212" t="n"/>
     </row>
     <row r="45" ht="15" customHeight="1" s="104">
       <c r="A45" s="109" t="inlineStr">
@@ -1926,8 +2045,8 @@
           <t>Mortgage Payable - Building</t>
         </is>
       </c>
-      <c r="C45" s="112" t="n"/>
-      <c r="D45" s="111" t="n"/>
+      <c r="C45" s="213" t="n"/>
+      <c r="D45" s="212" t="n"/>
     </row>
     <row r="46" ht="15" customHeight="1" s="104">
       <c r="A46" s="109" t="inlineStr">
@@ -1940,8 +2059,8 @@
           <t>Mortgage Payable - Nonrecourse portion</t>
         </is>
       </c>
-      <c r="C46" s="112" t="n"/>
-      <c r="D46" s="111" t="n"/>
+      <c r="C46" s="213" t="n"/>
+      <c r="D46" s="212" t="n"/>
     </row>
     <row r="47" ht="15" customHeight="1" s="104">
       <c r="A47" s="109" t="inlineStr">
@@ -1954,8 +2073,8 @@
           <t>Loans from Partners</t>
         </is>
       </c>
-      <c r="C47" s="112" t="n"/>
-      <c r="D47" s="111" t="n"/>
+      <c r="C47" s="213" t="n"/>
+      <c r="D47" s="212" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1" s="104">
       <c r="A48" s="109" t="inlineStr">
@@ -1968,11 +2087,11 @@
           <t>Other Long-term Liabilities</t>
         </is>
       </c>
-      <c r="C48" s="112" t="n"/>
-      <c r="D48" s="111" t="n"/>
+      <c r="C48" s="213" t="n"/>
+      <c r="D48" s="212" t="n"/>
     </row>
     <row r="49" ht="21.75" customHeight="1" s="104">
-      <c r="A49" s="108" t="inlineStr">
+      <c r="A49" s="211" t="inlineStr">
         <is>
           <t>PARTNERS' EQUITY</t>
         </is>
@@ -1992,8 +2111,8 @@
           <t>Partner A - Capital Account (Beg Bal - MUST = PY Ending)</t>
         </is>
       </c>
-      <c r="C50" s="112" t="n"/>
-      <c r="D50" s="111" t="n"/>
+      <c r="C50" s="213" t="n"/>
+      <c r="D50" s="212" t="n"/>
     </row>
     <row r="51" ht="15" customHeight="1" s="104">
       <c r="A51" s="113" t="inlineStr">
@@ -2006,8 +2125,8 @@
           <t>Partner B - Capital Account (Beg Bal - MUST = PY Ending)</t>
         </is>
       </c>
-      <c r="C51" s="112" t="n"/>
-      <c r="D51" s="111" t="n"/>
+      <c r="C51" s="213" t="n"/>
+      <c r="D51" s="212" t="n"/>
     </row>
     <row r="52" ht="15" customHeight="1" s="104">
       <c r="A52" s="109" t="inlineStr">
@@ -2020,8 +2139,8 @@
           <t>Partner A - Draws/Distributions</t>
         </is>
       </c>
-      <c r="C52" s="111" t="n"/>
-      <c r="D52" s="112" t="n"/>
+      <c r="C52" s="212" t="n"/>
+      <c r="D52" s="213" t="n"/>
     </row>
     <row r="53" ht="15" customHeight="1" s="104">
       <c r="A53" s="109" t="inlineStr">
@@ -2034,8 +2153,8 @@
           <t>Partner B - Draws/Distributions</t>
         </is>
       </c>
-      <c r="C53" s="111" t="n"/>
-      <c r="D53" s="112" t="n"/>
+      <c r="C53" s="212" t="n"/>
+      <c r="D53" s="213" t="n"/>
     </row>
     <row r="54" ht="15" customHeight="1" s="104">
       <c r="A54" s="109" t="inlineStr">
@@ -2048,8 +2167,8 @@
           <t>Partner A - Contributions</t>
         </is>
       </c>
-      <c r="C54" s="112" t="n"/>
-      <c r="D54" s="111" t="n"/>
+      <c r="C54" s="213" t="n"/>
+      <c r="D54" s="212" t="n"/>
     </row>
     <row r="55" ht="15" customHeight="1" s="104">
       <c r="A55" s="109" t="inlineStr">
@@ -2062,11 +2181,11 @@
           <t>Partner B - Contributions</t>
         </is>
       </c>
-      <c r="C55" s="112" t="n"/>
-      <c r="D55" s="111" t="n"/>
+      <c r="C55" s="213" t="n"/>
+      <c r="D55" s="212" t="n"/>
     </row>
     <row r="56" ht="21.75" customHeight="1" s="104">
-      <c r="A56" s="108" t="inlineStr">
+      <c r="A56" s="211" t="inlineStr">
         <is>
           <t>REVENUE</t>
         </is>
@@ -2086,8 +2205,8 @@
           <t>Gross Sales / Revenue</t>
         </is>
       </c>
-      <c r="C57" s="112" t="n"/>
-      <c r="D57" s="111" t="n"/>
+      <c r="C57" s="213" t="n"/>
+      <c r="D57" s="212" t="n"/>
     </row>
     <row r="58" ht="15" customHeight="1" s="104">
       <c r="A58" s="109" t="inlineStr">
@@ -2100,8 +2219,8 @@
           <t>Sales Returns &amp; Allowances</t>
         </is>
       </c>
-      <c r="C58" s="111" t="n"/>
-      <c r="D58" s="112" t="n"/>
+      <c r="C58" s="212" t="n"/>
+      <c r="D58" s="213" t="n"/>
     </row>
     <row r="59" ht="15" customHeight="1" s="104">
       <c r="A59" s="109" t="inlineStr">
@@ -2114,8 +2233,8 @@
           <t>Rental Income - Real Estate (Form 8825)</t>
         </is>
       </c>
-      <c r="C59" s="112" t="n"/>
-      <c r="D59" s="111" t="n"/>
+      <c r="C59" s="213" t="n"/>
+      <c r="D59" s="212" t="n"/>
     </row>
     <row r="60" ht="15" customHeight="1" s="104">
       <c r="A60" s="109" t="inlineStr">
@@ -2128,8 +2247,8 @@
           <t>Rental Income - Equipment</t>
         </is>
       </c>
-      <c r="C60" s="112" t="n"/>
-      <c r="D60" s="111" t="n"/>
+      <c r="C60" s="213" t="n"/>
+      <c r="D60" s="212" t="n"/>
     </row>
     <row r="61" ht="15" customHeight="1" s="104">
       <c r="A61" s="109" t="inlineStr">
@@ -2142,8 +2261,8 @@
           <t>Interest Income - Bank</t>
         </is>
       </c>
-      <c r="C61" s="112" t="n"/>
-      <c r="D61" s="111" t="n"/>
+      <c r="C61" s="213" t="n"/>
+      <c r="D61" s="212" t="n"/>
     </row>
     <row r="62" ht="15" customHeight="1" s="104">
       <c r="A62" s="109" t="inlineStr">
@@ -2156,8 +2275,8 @@
           <t>Interest Income - Municipal Bonds (Tax-Exempt)</t>
         </is>
       </c>
-      <c r="C62" s="112" t="n"/>
-      <c r="D62" s="111" t="n"/>
+      <c r="C62" s="213" t="n"/>
+      <c r="D62" s="212" t="n"/>
     </row>
     <row r="63" ht="15" customHeight="1" s="104">
       <c r="A63" s="109" t="inlineStr">
@@ -2170,8 +2289,8 @@
           <t>Interest Income - Corporate Bonds</t>
         </is>
       </c>
-      <c r="C63" s="112" t="n"/>
-      <c r="D63" s="111" t="n"/>
+      <c r="C63" s="213" t="n"/>
+      <c r="D63" s="212" t="n"/>
     </row>
     <row r="64" ht="15" customHeight="1" s="104">
       <c r="A64" s="109" t="inlineStr">
@@ -2184,8 +2303,8 @@
           <t>Dividend Income - Ordinary</t>
         </is>
       </c>
-      <c r="C64" s="112" t="n"/>
-      <c r="D64" s="111" t="n"/>
+      <c r="C64" s="213" t="n"/>
+      <c r="D64" s="212" t="n"/>
     </row>
     <row r="65" ht="15" customHeight="1" s="104">
       <c r="A65" s="109" t="inlineStr">
@@ -2198,8 +2317,8 @@
           <t>Dividend Income - Qualified</t>
         </is>
       </c>
-      <c r="C65" s="112" t="n"/>
-      <c r="D65" s="111" t="n"/>
+      <c r="C65" s="213" t="n"/>
+      <c r="D65" s="212" t="n"/>
     </row>
     <row r="66" ht="15" customHeight="1" s="104">
       <c r="A66" s="109" t="inlineStr">
@@ -2212,8 +2331,8 @@
           <t>Royalty Income</t>
         </is>
       </c>
-      <c r="C66" s="112" t="n"/>
-      <c r="D66" s="111" t="n"/>
+      <c r="C66" s="213" t="n"/>
+      <c r="D66" s="212" t="n"/>
     </row>
     <row r="67" ht="15" customHeight="1" s="104">
       <c r="A67" s="109" t="inlineStr">
@@ -2226,8 +2345,8 @@
           <t>Gain on Sale of Equipment (Sec 1231 - held &gt;1yr)</t>
         </is>
       </c>
-      <c r="C67" s="112" t="n"/>
-      <c r="D67" s="111" t="n"/>
+      <c r="C67" s="213" t="n"/>
+      <c r="D67" s="212" t="n"/>
     </row>
     <row r="68" ht="15" customHeight="1" s="104">
       <c r="A68" s="109" t="inlineStr">
@@ -2240,8 +2359,8 @@
           <t>Gain on Sale of Stock - Short-term</t>
         </is>
       </c>
-      <c r="C68" s="112" t="n"/>
-      <c r="D68" s="111" t="n"/>
+      <c r="C68" s="213" t="n"/>
+      <c r="D68" s="212" t="n"/>
     </row>
     <row r="69" ht="15" customHeight="1" s="104">
       <c r="A69" s="109" t="inlineStr">
@@ -2254,8 +2373,8 @@
           <t>Gain on Sale of Stock - Long-term</t>
         </is>
       </c>
-      <c r="C69" s="112" t="n"/>
-      <c r="D69" s="111" t="n"/>
+      <c r="C69" s="213" t="n"/>
+      <c r="D69" s="212" t="n"/>
     </row>
     <row r="70" ht="15" customHeight="1" s="104">
       <c r="A70" s="109" t="inlineStr">
@@ -2268,8 +2387,8 @@
           <t>Gain on Sale of Collectibles (Art)</t>
         </is>
       </c>
-      <c r="C70" s="112" t="n"/>
-      <c r="D70" s="111" t="n"/>
+      <c r="C70" s="213" t="n"/>
+      <c r="D70" s="212" t="n"/>
     </row>
     <row r="71" ht="15" customHeight="1" s="104">
       <c r="A71" s="109" t="inlineStr">
@@ -2282,8 +2401,8 @@
           <t>Income from Sub-Partnership (K-1 ordinary)</t>
         </is>
       </c>
-      <c r="C71" s="112" t="n"/>
-      <c r="D71" s="111" t="n"/>
+      <c r="C71" s="213" t="n"/>
+      <c r="D71" s="212" t="n"/>
     </row>
     <row r="72" ht="15" customHeight="1" s="104">
       <c r="A72" s="109" t="inlineStr">
@@ -2296,8 +2415,8 @@
           <t>Income from Sub-Partnership (K-1 separately stated - LTCG)</t>
         </is>
       </c>
-      <c r="C72" s="112" t="n"/>
-      <c r="D72" s="111" t="n"/>
+      <c r="C72" s="213" t="n"/>
+      <c r="D72" s="212" t="n"/>
     </row>
     <row r="73" ht="15" customHeight="1" s="104">
       <c r="A73" s="109" t="inlineStr">
@@ -2310,8 +2429,8 @@
           <t>Cancellation of Debt Income</t>
         </is>
       </c>
-      <c r="C73" s="112" t="n"/>
-      <c r="D73" s="111" t="n"/>
+      <c r="C73" s="213" t="n"/>
+      <c r="D73" s="212" t="n"/>
     </row>
     <row r="74" ht="15" customHeight="1" s="104">
       <c r="A74" s="109" t="inlineStr">
@@ -2324,11 +2443,11 @@
           <t>Other Miscellaneous Income</t>
         </is>
       </c>
-      <c r="C74" s="112" t="n"/>
-      <c r="D74" s="111" t="n"/>
+      <c r="C74" s="213" t="n"/>
+      <c r="D74" s="212" t="n"/>
     </row>
     <row r="75" ht="21.75" customHeight="1" s="104">
-      <c r="A75" s="108" t="inlineStr">
+      <c r="A75" s="211" t="inlineStr">
         <is>
           <t>COST OF GOODS SOLD</t>
         </is>
@@ -2348,8 +2467,8 @@
           <t>Beginning Inventory (MUST = PY Ending Inventory)</t>
         </is>
       </c>
-      <c r="C76" s="111" t="n"/>
-      <c r="D76" s="112" t="n"/>
+      <c r="C76" s="212" t="n"/>
+      <c r="D76" s="213" t="n"/>
     </row>
     <row r="77" ht="15" customHeight="1" s="104">
       <c r="A77" s="109" t="inlineStr">
@@ -2362,8 +2481,8 @@
           <t>Purchases</t>
         </is>
       </c>
-      <c r="C77" s="111" t="n"/>
-      <c r="D77" s="112" t="n"/>
+      <c r="C77" s="212" t="n"/>
+      <c r="D77" s="213" t="n"/>
     </row>
     <row r="78" ht="15" customHeight="1" s="104">
       <c r="A78" s="109" t="inlineStr">
@@ -2376,8 +2495,8 @@
           <t>Direct Labor</t>
         </is>
       </c>
-      <c r="C78" s="111" t="n"/>
-      <c r="D78" s="112" t="n"/>
+      <c r="C78" s="212" t="n"/>
+      <c r="D78" s="213" t="n"/>
     </row>
     <row r="79" ht="15" customHeight="1" s="104">
       <c r="A79" s="109" t="inlineStr">
@@ -2390,8 +2509,8 @@
           <t>Freight-In</t>
         </is>
       </c>
-      <c r="C79" s="111" t="n"/>
-      <c r="D79" s="112" t="n"/>
+      <c r="C79" s="212" t="n"/>
+      <c r="D79" s="213" t="n"/>
     </row>
     <row r="80" ht="15" customHeight="1" s="104">
       <c r="A80" s="109" t="inlineStr">
@@ -2404,8 +2523,8 @@
           <t>Depreciation in COGS (manufacturing equip)</t>
         </is>
       </c>
-      <c r="C80" s="111" t="n"/>
-      <c r="D80" s="112" t="n"/>
+      <c r="C80" s="212" t="n"/>
+      <c r="D80" s="213" t="n"/>
     </row>
     <row r="81" ht="15" customHeight="1" s="104">
       <c r="A81" s="109" t="inlineStr">
@@ -2418,8 +2537,8 @@
           <t>Other Manufacturing Overhead</t>
         </is>
       </c>
-      <c r="C81" s="111" t="n"/>
-      <c r="D81" s="112" t="n"/>
+      <c r="C81" s="212" t="n"/>
+      <c r="D81" s="213" t="n"/>
     </row>
     <row r="82" ht="15" customHeight="1" s="104">
       <c r="A82" s="109" t="inlineStr">
@@ -2432,11 +2551,11 @@
           <t>Less: Ending Inventory</t>
         </is>
       </c>
-      <c r="C82" s="112" t="n"/>
-      <c r="D82" s="111" t="n"/>
+      <c r="C82" s="213" t="n"/>
+      <c r="D82" s="212" t="n"/>
     </row>
     <row r="83" ht="21.75" customHeight="1" s="104">
-      <c r="A83" s="108" t="inlineStr">
+      <c r="A83" s="211" t="inlineStr">
         <is>
           <t>OPERATING EXPENSES</t>
         </is>
@@ -2456,8 +2575,8 @@
           <t>Salaries &amp; Wages (W-2 employees)</t>
         </is>
       </c>
-      <c r="C84" s="111" t="n"/>
-      <c r="D84" s="112" t="n"/>
+      <c r="C84" s="212" t="n"/>
+      <c r="D84" s="213" t="n"/>
     </row>
     <row r="85" ht="15" customHeight="1" s="104">
       <c r="A85" s="109" t="inlineStr">
@@ -2470,8 +2589,8 @@
           <t>Guaranteed Payments - Partner A (services)</t>
         </is>
       </c>
-      <c r="C85" s="111" t="n"/>
-      <c r="D85" s="112" t="n"/>
+      <c r="C85" s="212" t="n"/>
+      <c r="D85" s="213" t="n"/>
     </row>
     <row r="86" ht="15" customHeight="1" s="104">
       <c r="A86" s="109" t="inlineStr">
@@ -2484,8 +2603,8 @@
           <t>Guaranteed Payments - Partner B (services)</t>
         </is>
       </c>
-      <c r="C86" s="111" t="n"/>
-      <c r="D86" s="112" t="n"/>
+      <c r="C86" s="212" t="n"/>
+      <c r="D86" s="213" t="n"/>
     </row>
     <row r="87" ht="15" customHeight="1" s="104">
       <c r="A87" s="109" t="inlineStr">
@@ -2498,8 +2617,8 @@
           <t>Guaranteed Payments - Use of Capital</t>
         </is>
       </c>
-      <c r="C87" s="111" t="n"/>
-      <c r="D87" s="112" t="n"/>
+      <c r="C87" s="212" t="n"/>
+      <c r="D87" s="213" t="n"/>
     </row>
     <row r="88" ht="15" customHeight="1" s="104">
       <c r="A88" s="109" t="inlineStr">
@@ -2512,8 +2631,8 @@
           <t>Payroll Taxes (employer portion)</t>
         </is>
       </c>
-      <c r="C88" s="111" t="n"/>
-      <c r="D88" s="112" t="n"/>
+      <c r="C88" s="212" t="n"/>
+      <c r="D88" s="213" t="n"/>
     </row>
     <row r="89" ht="15" customHeight="1" s="104">
       <c r="A89" s="109" t="inlineStr">
@@ -2526,8 +2645,8 @@
           <t>Employee Health Insurance</t>
         </is>
       </c>
-      <c r="C89" s="111" t="n"/>
-      <c r="D89" s="112" t="n"/>
+      <c r="C89" s="212" t="n"/>
+      <c r="D89" s="213" t="n"/>
     </row>
     <row r="90" ht="15" customHeight="1" s="104">
       <c r="A90" s="109" t="inlineStr">
@@ -2540,8 +2659,8 @@
           <t>Partner Health Insurance (Partner A)</t>
         </is>
       </c>
-      <c r="C90" s="111" t="n"/>
-      <c r="D90" s="112" t="n"/>
+      <c r="C90" s="212" t="n"/>
+      <c r="D90" s="213" t="n"/>
     </row>
     <row r="91" ht="15" customHeight="1" s="104">
       <c r="A91" s="109" t="inlineStr">
@@ -2554,8 +2673,8 @@
           <t>Partner Health Insurance (Partner B)</t>
         </is>
       </c>
-      <c r="C91" s="111" t="n"/>
-      <c r="D91" s="112" t="n"/>
+      <c r="C91" s="212" t="n"/>
+      <c r="D91" s="213" t="n"/>
     </row>
     <row r="92" ht="15" customHeight="1" s="104">
       <c r="A92" s="109" t="inlineStr">
@@ -2568,8 +2687,8 @@
           <t>401(k) Employer Match</t>
         </is>
       </c>
-      <c r="C92" s="111" t="n"/>
-      <c r="D92" s="112" t="n"/>
+      <c r="C92" s="212" t="n"/>
+      <c r="D92" s="213" t="n"/>
     </row>
     <row r="93" ht="15" customHeight="1" s="104">
       <c r="A93" s="109" t="inlineStr">
@@ -2582,8 +2701,8 @@
           <t>Workers Compensation Insurance</t>
         </is>
       </c>
-      <c r="C93" s="111" t="n"/>
-      <c r="D93" s="112" t="n"/>
+      <c r="C93" s="212" t="n"/>
+      <c r="D93" s="213" t="n"/>
     </row>
     <row r="94" ht="15" customHeight="1" s="104">
       <c r="A94" s="109" t="inlineStr">
@@ -2596,8 +2715,8 @@
           <t>Rent - Office Space</t>
         </is>
       </c>
-      <c r="C94" s="111" t="n"/>
-      <c r="D94" s="112" t="n"/>
+      <c r="C94" s="212" t="n"/>
+      <c r="D94" s="213" t="n"/>
     </row>
     <row r="95" ht="15" customHeight="1" s="104">
       <c r="A95" s="109" t="inlineStr">
@@ -2610,8 +2729,8 @@
           <t>Rent - Equipment</t>
         </is>
       </c>
-      <c r="C95" s="111" t="n"/>
-      <c r="D95" s="112" t="n"/>
+      <c r="C95" s="212" t="n"/>
+      <c r="D95" s="213" t="n"/>
     </row>
     <row r="96" ht="15" customHeight="1" s="104">
       <c r="A96" s="109" t="inlineStr">
@@ -2624,8 +2743,8 @@
           <t>Repairs &amp; Maintenance</t>
         </is>
       </c>
-      <c r="C96" s="111" t="n"/>
-      <c r="D96" s="112" t="n"/>
+      <c r="C96" s="212" t="n"/>
+      <c r="D96" s="213" t="n"/>
     </row>
     <row r="97" ht="15" customHeight="1" s="104">
       <c r="A97" s="109" t="inlineStr">
@@ -2638,8 +2757,8 @@
           <t>Capital Improvement (Expensed on Books - should be capitalized)</t>
         </is>
       </c>
-      <c r="C97" s="111" t="n"/>
-      <c r="D97" s="112" t="n"/>
+      <c r="C97" s="212" t="n"/>
+      <c r="D97" s="213" t="n"/>
     </row>
     <row r="98" ht="15" customHeight="1" s="104">
       <c r="A98" s="109" t="inlineStr">
@@ -2652,8 +2771,8 @@
           <t>Depreciation - Book</t>
         </is>
       </c>
-      <c r="C98" s="111" t="n"/>
-      <c r="D98" s="112" t="n"/>
+      <c r="C98" s="212" t="n"/>
+      <c r="D98" s="213" t="n"/>
     </row>
     <row r="99" ht="15" customHeight="1" s="104">
       <c r="A99" s="109" t="inlineStr">
@@ -2666,8 +2785,8 @@
           <t>Amortization - Goodwill (Book - 10yr)</t>
         </is>
       </c>
-      <c r="C99" s="111" t="n"/>
-      <c r="D99" s="112" t="n"/>
+      <c r="C99" s="212" t="n"/>
+      <c r="D99" s="213" t="n"/>
     </row>
     <row r="100" ht="15" customHeight="1" s="104">
       <c r="A100" s="109" t="inlineStr">
@@ -2680,8 +2799,8 @@
           <t>Amortization - Patents (Book - 10yr)</t>
         </is>
       </c>
-      <c r="C100" s="111" t="n"/>
-      <c r="D100" s="112" t="n"/>
+      <c r="C100" s="212" t="n"/>
+      <c r="D100" s="213" t="n"/>
     </row>
     <row r="101" ht="15" customHeight="1" s="104">
       <c r="A101" s="109" t="inlineStr">
@@ -2694,8 +2813,8 @@
           <t>Utilities</t>
         </is>
       </c>
-      <c r="C101" s="111" t="n"/>
-      <c r="D101" s="112" t="n"/>
+      <c r="C101" s="212" t="n"/>
+      <c r="D101" s="213" t="n"/>
     </row>
     <row r="102" ht="15" customHeight="1" s="104">
       <c r="A102" s="109" t="inlineStr">
@@ -2708,8 +2827,8 @@
           <t>Telephone &amp; Internet</t>
         </is>
       </c>
-      <c r="C102" s="111" t="n"/>
-      <c r="D102" s="112" t="n"/>
+      <c r="C102" s="212" t="n"/>
+      <c r="D102" s="213" t="n"/>
     </row>
     <row r="103" ht="15" customHeight="1" s="104">
       <c r="A103" s="109" t="inlineStr">
@@ -2722,8 +2841,8 @@
           <t>Office Supplies</t>
         </is>
       </c>
-      <c r="C103" s="111" t="n"/>
-      <c r="D103" s="112" t="n"/>
+      <c r="C103" s="212" t="n"/>
+      <c r="D103" s="213" t="n"/>
     </row>
     <row r="104" ht="15" customHeight="1" s="104">
       <c r="A104" s="109" t="inlineStr">
@@ -2736,8 +2855,8 @@
           <t>Postage &amp; Shipping</t>
         </is>
       </c>
-      <c r="C104" s="111" t="n"/>
-      <c r="D104" s="112" t="n"/>
+      <c r="C104" s="212" t="n"/>
+      <c r="D104" s="213" t="n"/>
     </row>
     <row r="105" ht="15" customHeight="1" s="104">
       <c r="A105" s="109" t="inlineStr">
@@ -2750,8 +2869,8 @@
           <t>Business Insurance (GL, E&amp;O)</t>
         </is>
       </c>
-      <c r="C105" s="111" t="n"/>
-      <c r="D105" s="112" t="n"/>
+      <c r="C105" s="212" t="n"/>
+      <c r="D105" s="213" t="n"/>
     </row>
     <row r="106" ht="15" customHeight="1" s="104">
       <c r="A106" s="109" t="inlineStr">
@@ -2764,8 +2883,8 @@
           <t>Professional Fees - Accounting</t>
         </is>
       </c>
-      <c r="C106" s="111" t="n"/>
-      <c r="D106" s="112" t="n"/>
+      <c r="C106" s="212" t="n"/>
+      <c r="D106" s="213" t="n"/>
     </row>
     <row r="107" ht="15" customHeight="1" s="104">
       <c r="A107" s="109" t="inlineStr">
@@ -2778,8 +2897,8 @@
           <t>Professional Fees - Legal</t>
         </is>
       </c>
-      <c r="C107" s="111" t="n"/>
-      <c r="D107" s="112" t="n"/>
+      <c r="C107" s="212" t="n"/>
+      <c r="D107" s="213" t="n"/>
     </row>
     <row r="108" ht="15" customHeight="1" s="104">
       <c r="A108" s="109" t="inlineStr">
@@ -2792,8 +2911,8 @@
           <t>Professional Fees - Consulting</t>
         </is>
       </c>
-      <c r="C108" s="111" t="n"/>
-      <c r="D108" s="112" t="n"/>
+      <c r="C108" s="212" t="n"/>
+      <c r="D108" s="213" t="n"/>
     </row>
     <row r="109" ht="15" customHeight="1" s="104">
       <c r="A109" s="109" t="inlineStr">
@@ -2806,8 +2925,8 @@
           <t>Advertising &amp; Marketing</t>
         </is>
       </c>
-      <c r="C109" s="111" t="n"/>
-      <c r="D109" s="112" t="n"/>
+      <c r="C109" s="212" t="n"/>
+      <c r="D109" s="213" t="n"/>
     </row>
     <row r="110" ht="15" customHeight="1" s="104">
       <c r="A110" s="109" t="inlineStr">
@@ -2820,8 +2939,8 @@
           <t>Travel Expense</t>
         </is>
       </c>
-      <c r="C110" s="111" t="n"/>
-      <c r="D110" s="112" t="n"/>
+      <c r="C110" s="212" t="n"/>
+      <c r="D110" s="213" t="n"/>
     </row>
     <row r="111" ht="15" customHeight="1" s="104">
       <c r="A111" s="109" t="inlineStr">
@@ -2834,8 +2953,8 @@
           <t>Business Meals (100% on books)</t>
         </is>
       </c>
-      <c r="C111" s="111" t="n"/>
-      <c r="D111" s="112" t="n"/>
+      <c r="C111" s="212" t="n"/>
+      <c r="D111" s="213" t="n"/>
     </row>
     <row r="112" ht="15" customHeight="1" s="104">
       <c r="A112" s="109" t="inlineStr">
@@ -2848,8 +2967,8 @@
           <t>Entertainment</t>
         </is>
       </c>
-      <c r="C112" s="111" t="n"/>
-      <c r="D112" s="112" t="n"/>
+      <c r="C112" s="212" t="n"/>
+      <c r="D112" s="213" t="n"/>
     </row>
     <row r="113" ht="15" customHeight="1" s="104">
       <c r="A113" s="109" t="inlineStr">
@@ -2862,8 +2981,8 @@
           <t>Club Dues (Country Club)</t>
         </is>
       </c>
-      <c r="C113" s="111" t="n"/>
-      <c r="D113" s="112" t="n"/>
+      <c r="C113" s="212" t="n"/>
+      <c r="D113" s="213" t="n"/>
     </row>
     <row r="114" ht="15" customHeight="1" s="104">
       <c r="A114" s="109" t="inlineStr">
@@ -2876,8 +2995,8 @@
           <t>Auto Expense (non-depreciation)</t>
         </is>
       </c>
-      <c r="C114" s="111" t="n"/>
-      <c r="D114" s="112" t="n"/>
+      <c r="C114" s="212" t="n"/>
+      <c r="D114" s="213" t="n"/>
     </row>
     <row r="115" ht="15" customHeight="1" s="104">
       <c r="A115" s="109" t="inlineStr">
@@ -2890,8 +3009,8 @@
           <t>Charitable Contributions</t>
         </is>
       </c>
-      <c r="C115" s="111" t="n"/>
-      <c r="D115" s="112" t="n"/>
+      <c r="C115" s="212" t="n"/>
+      <c r="D115" s="213" t="n"/>
     </row>
     <row r="116" ht="15" customHeight="1" s="104">
       <c r="A116" s="109" t="inlineStr">
@@ -2904,8 +3023,8 @@
           <t>Penalties &amp; Fines</t>
         </is>
       </c>
-      <c r="C116" s="111" t="n"/>
-      <c r="D116" s="112" t="n"/>
+      <c r="C116" s="212" t="n"/>
+      <c r="D116" s="213" t="n"/>
     </row>
     <row r="117" ht="15" customHeight="1" s="104">
       <c r="A117" s="109" t="inlineStr">
@@ -2918,8 +3037,8 @@
           <t>Political Contributions</t>
         </is>
       </c>
-      <c r="C117" s="111" t="n"/>
-      <c r="D117" s="112" t="n"/>
+      <c r="C117" s="212" t="n"/>
+      <c r="D117" s="213" t="n"/>
     </row>
     <row r="118" ht="15" customHeight="1" s="104">
       <c r="A118" s="109" t="inlineStr">
@@ -2932,8 +3051,8 @@
           <t>Interest Expense - Business Line of Credit</t>
         </is>
       </c>
-      <c r="C118" s="111" t="n"/>
-      <c r="D118" s="112" t="n"/>
+      <c r="C118" s="212" t="n"/>
+      <c r="D118" s="213" t="n"/>
     </row>
     <row r="119" ht="15" customHeight="1" s="104">
       <c r="A119" s="109" t="inlineStr">
@@ -2946,8 +3065,8 @@
           <t>Interest Expense - Mortgage</t>
         </is>
       </c>
-      <c r="C119" s="111" t="n"/>
-      <c r="D119" s="112" t="n"/>
+      <c r="C119" s="212" t="n"/>
+      <c r="D119" s="213" t="n"/>
     </row>
     <row r="120" ht="15" customHeight="1" s="104">
       <c r="A120" s="109" t="inlineStr">
@@ -2960,8 +3079,8 @@
           <t>Interest Expense - Investment Margin Account</t>
         </is>
       </c>
-      <c r="C120" s="111" t="n"/>
-      <c r="D120" s="112" t="n"/>
+      <c r="C120" s="212" t="n"/>
+      <c r="D120" s="213" t="n"/>
     </row>
     <row r="121" ht="15" customHeight="1" s="104">
       <c r="A121" s="109" t="inlineStr">
@@ -2974,8 +3093,8 @@
           <t>Taxes - Property</t>
         </is>
       </c>
-      <c r="C121" s="111" t="n"/>
-      <c r="D121" s="112" t="n"/>
+      <c r="C121" s="212" t="n"/>
+      <c r="D121" s="213" t="n"/>
     </row>
     <row r="122" ht="15" customHeight="1" s="104">
       <c r="A122" s="109" t="inlineStr">
@@ -2988,8 +3107,8 @@
           <t>Taxes - State Franchise/Income</t>
         </is>
       </c>
-      <c r="C122" s="111" t="n"/>
-      <c r="D122" s="112" t="n"/>
+      <c r="C122" s="212" t="n"/>
+      <c r="D122" s="213" t="n"/>
     </row>
     <row r="123" ht="15" customHeight="1" s="104">
       <c r="A123" s="109" t="inlineStr">
@@ -3002,8 +3121,8 @@
           <t>Taxes - Business Licenses</t>
         </is>
       </c>
-      <c r="C123" s="111" t="n"/>
-      <c r="D123" s="112" t="n"/>
+      <c r="C123" s="212" t="n"/>
+      <c r="D123" s="213" t="n"/>
     </row>
     <row r="124" ht="15" customHeight="1" s="104">
       <c r="A124" s="109" t="inlineStr">
@@ -3016,8 +3135,8 @@
           <t>Bad Debt Expense (Reserve Method on Books)</t>
         </is>
       </c>
-      <c r="C124" s="111" t="n"/>
-      <c r="D124" s="112" t="n"/>
+      <c r="C124" s="212" t="n"/>
+      <c r="D124" s="213" t="n"/>
     </row>
     <row r="125" ht="15" customHeight="1" s="104">
       <c r="A125" s="109" t="inlineStr">
@@ -3030,8 +3149,8 @@
           <t>Warranty Reserve Expense</t>
         </is>
       </c>
-      <c r="C125" s="111" t="n"/>
-      <c r="D125" s="112" t="n"/>
+      <c r="C125" s="212" t="n"/>
+      <c r="D125" s="213" t="n"/>
     </row>
     <row r="126" ht="15" customHeight="1" s="104">
       <c r="A126" s="109" t="inlineStr">
@@ -3044,8 +3163,8 @@
           <t>Litigation Reserve Expense</t>
         </is>
       </c>
-      <c r="C126" s="111" t="n"/>
-      <c r="D126" s="112" t="n"/>
+      <c r="C126" s="212" t="n"/>
+      <c r="D126" s="213" t="n"/>
     </row>
     <row r="127" ht="15" customHeight="1" s="104">
       <c r="A127" s="109" t="inlineStr">
@@ -3058,8 +3177,8 @@
           <t>Life Insurance Premiums (Key Person - Partnership Beneficiary)</t>
         </is>
       </c>
-      <c r="C127" s="111" t="n"/>
-      <c r="D127" s="112" t="n"/>
+      <c r="C127" s="212" t="n"/>
+      <c r="D127" s="213" t="n"/>
     </row>
     <row r="128" ht="15" customHeight="1" s="104">
       <c r="A128" s="109" t="inlineStr">
@@ -3072,11 +3191,11 @@
           <t>Miscellaneous Expense</t>
         </is>
       </c>
-      <c r="C128" s="111" t="n"/>
-      <c r="D128" s="112" t="n"/>
+      <c r="C128" s="212" t="n"/>
+      <c r="D128" s="213" t="n"/>
     </row>
     <row r="129" ht="21.75" customHeight="1" s="104">
-      <c r="A129" s="108" t="inlineStr">
+      <c r="A129" s="211" t="inlineStr">
         <is>
           <t>RENTAL PROPERTY EXPENSES (Form 8825)</t>
         </is>
@@ -3096,8 +3215,8 @@
           <t>Rental Property - Depreciation (Book)</t>
         </is>
       </c>
-      <c r="C130" s="111" t="n"/>
-      <c r="D130" s="112" t="n"/>
+      <c r="C130" s="212" t="n"/>
+      <c r="D130" s="213" t="n"/>
     </row>
     <row r="131" ht="15" customHeight="1" s="104">
       <c r="A131" s="109" t="inlineStr">
@@ -3110,8 +3229,8 @@
           <t>Rental Property - Insurance</t>
         </is>
       </c>
-      <c r="C131" s="111" t="n"/>
-      <c r="D131" s="112" t="n"/>
+      <c r="C131" s="212" t="n"/>
+      <c r="D131" s="213" t="n"/>
     </row>
     <row r="132" ht="15" customHeight="1" s="104">
       <c r="A132" s="109" t="inlineStr">
@@ -3124,8 +3243,8 @@
           <t>Rental Property - Repairs &amp; Maintenance</t>
         </is>
       </c>
-      <c r="C132" s="111" t="n"/>
-      <c r="D132" s="112" t="n"/>
+      <c r="C132" s="212" t="n"/>
+      <c r="D132" s="213" t="n"/>
     </row>
     <row r="133" ht="15" customHeight="1" s="104">
       <c r="A133" s="109" t="inlineStr">
@@ -3138,8 +3257,8 @@
           <t>Rental Property - Property Taxes</t>
         </is>
       </c>
-      <c r="C133" s="111" t="n"/>
-      <c r="D133" s="112" t="n"/>
+      <c r="C133" s="212" t="n"/>
+      <c r="D133" s="213" t="n"/>
     </row>
     <row r="134" ht="15" customHeight="1" s="104">
       <c r="A134" s="109" t="inlineStr">
@@ -3152,8 +3271,8 @@
           <t>Rental Property - Mortgage Interest</t>
         </is>
       </c>
-      <c r="C134" s="111" t="n"/>
-      <c r="D134" s="112" t="n"/>
+      <c r="C134" s="212" t="n"/>
+      <c r="D134" s="213" t="n"/>
     </row>
     <row r="135" ht="15" customHeight="1" s="104">
       <c r="A135" s="109" t="inlineStr">
@@ -3166,8 +3285,8 @@
           <t>Rental Property - Utilities</t>
         </is>
       </c>
-      <c r="C135" s="111" t="n"/>
-      <c r="D135" s="112" t="n"/>
+      <c r="C135" s="212" t="n"/>
+      <c r="D135" s="213" t="n"/>
     </row>
     <row r="136" ht="15" customHeight="1" s="104">
       <c r="A136" s="109" t="inlineStr">
@@ -3180,26 +3299,28 @@
           <t>Rental Property - Management Fees</t>
         </is>
       </c>
-      <c r="C136" s="111" t="n"/>
-      <c r="D136" s="112" t="n"/>
-    </row>
+      <c r="C136" s="212" t="n"/>
+      <c r="D136" s="213" t="n"/>
+    </row>
+    <row r="137"/>
     <row r="138" ht="15" customHeight="1" s="104">
-      <c r="A138" s="115" t="n"/>
+      <c r="A138" s="214" t="n"/>
       <c r="B138" s="115" t="inlineStr">
         <is>
           <t>TOTAL TRIAL BALANCE</t>
         </is>
       </c>
-      <c r="C138" s="116">
+      <c r="C138" s="215">
         <f>SUM(C5:C136)</f>
         <v/>
       </c>
-      <c r="D138" s="116">
+      <c r="D138" s="215">
         <f>SUM(D5:D136)</f>
         <v/>
       </c>
     </row>
     <row r="139" ht="15" customHeight="1" s="104">
+      <c r="A139" s="216" t="n"/>
       <c r="B139" s="117" t="inlineStr">
         <is>
           <t>DIFFERENCE (should be zero)</t>
@@ -3281,6 +3402,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="31.5" customHeight="1" s="104">
       <c r="A5" s="107" t="inlineStr">
         <is>
@@ -3334,7 +3456,7 @@
       </c>
     </row>
     <row r="6" ht="21.75" customHeight="1" s="104">
-      <c r="A6" s="108" t="inlineStr">
+      <c r="A6" s="211" t="inlineStr">
         <is>
           <t>BALANCE SHEET — ASSETS</t>
         </is>
@@ -3557,8 +3679,9 @@
       <c r="I12" s="128" t="n"/>
       <c r="J12" s="129" t="n"/>
     </row>
+    <row r="13"/>
     <row r="14" ht="21.75" customHeight="1" s="104">
-      <c r="A14" s="108" t="inlineStr">
+      <c r="A14" s="211" t="inlineStr">
         <is>
           <t>BALANCE SHEET — LIABILITIES</t>
         </is>
@@ -3609,8 +3732,9 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="21.75" customHeight="1" s="104">
-      <c r="A17" s="108" t="inlineStr">
+      <c r="A17" s="211" t="inlineStr">
         <is>
           <t>BALANCE SHEET — PARTNERS' EQUITY / CAPITAL</t>
         </is>
@@ -3825,8 +3949,9 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25" ht="21.75" customHeight="1" s="104">
-      <c r="A25" s="108" t="inlineStr">
+      <c r="A25" s="211" t="inlineStr">
         <is>
           <t>PAGE 1 — INCOME</t>
         </is>
@@ -4200,7 +4325,7 @@
       </c>
     </row>
     <row r="36" ht="21.75" customHeight="1" s="104">
-      <c r="A36" s="108" t="inlineStr">
+      <c r="A36" s="211" t="inlineStr">
         <is>
           <t>PAGE 1 — DEDUCTIONS</t>
         </is>
@@ -5336,8 +5461,9 @@
         </is>
       </c>
     </row>
+    <row r="68"/>
     <row r="69" ht="21.75" customHeight="1" s="104">
-      <c r="A69" s="108" t="inlineStr">
+      <c r="A69" s="211" t="inlineStr">
         <is>
           <t>SCHEDULE K — SEPARATELY STATED ITEMS</t>
         </is>
@@ -5805,6 +5931,7 @@
         </is>
       </c>
     </row>
+    <row r="83"/>
     <row r="84" ht="19.5" customHeight="1" s="104">
       <c r="A84" s="109" t="n">
         <v>49</v>
@@ -6083,8 +6210,9 @@
         </is>
       </c>
     </row>
+    <row r="92"/>
     <row r="93" ht="21.75" customHeight="1" s="104">
-      <c r="A93" s="108" t="inlineStr">
+      <c r="A93" s="211" t="inlineStr">
         <is>
           <t>SCHEDULE M-1 — BOOK TO TAX RECONCILIATION</t>
         </is>
@@ -6406,8 +6534,9 @@
         </is>
       </c>
     </row>
+    <row r="104"/>
     <row r="105" ht="21.75" customHeight="1" s="104">
-      <c r="A105" s="108" t="inlineStr">
+      <c r="A105" s="211" t="inlineStr">
         <is>
           <t>SCHEDULE M-2 — PARTNERS' CAPITAL ACCOUNTS</t>
         </is>
@@ -6720,8 +6849,9 @@
         </is>
       </c>
     </row>
+    <row r="115"/>
     <row r="116" ht="21.75" customHeight="1" s="104">
-      <c r="A116" s="108" t="inlineStr">
+      <c r="A116" s="211" t="inlineStr">
         <is>
           <t>SCHEDULE L — BALANCE SHEET TIE-OUTS</t>
         </is>
@@ -6827,7 +6957,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="104">
-      <c r="A1" s="105" t="inlineStr">
+      <c r="A1" s="217" t="inlineStr">
         <is>
           <t>SCHEDULE K — DETAILED WORKPAPER</t>
         </is>
@@ -6840,6 +6970,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="104">
       <c r="A4" s="107" t="inlineStr">
         <is>
@@ -6883,7 +7014,7 @@
       </c>
     </row>
     <row r="5" ht="21.75" customHeight="1" s="104">
-      <c r="A5" s="108" t="inlineStr">
+      <c r="A5" s="211" t="inlineStr">
         <is>
           <t>INCOME (K Lines 1-11)</t>
         </is>
@@ -7665,6 +7796,7 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
     <row r="29" ht="21.75" customHeight="1" s="104">
       <c r="A29" s="108" t="inlineStr">
         <is>
@@ -8239,7 +8371,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="104">
-      <c r="A1" s="105" t="inlineStr">
+      <c r="A1" s="217" t="inlineStr">
         <is>
           <t>SCHEDULE M-1 — BOOK-TO-TAX RECONCILIATION WORKPAPER</t>
         </is>
@@ -8252,6 +8384,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="104">
       <c r="A4" s="107" t="inlineStr">
         <is>
@@ -8300,7 +8433,7 @@
       </c>
     </row>
     <row r="5" ht="21.75" customHeight="1" s="104">
-      <c r="A5" s="108" t="inlineStr">
+      <c r="A5" s="211" t="inlineStr">
         <is>
           <t>M-1 RECONCILIATION — FORM LINES</t>
         </is>
@@ -8666,8 +8799,9 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="21.75" customHeight="1" s="104">
-      <c r="A17" s="108" t="inlineStr">
+      <c r="A17" s="211" t="inlineStr">
         <is>
           <t>M-1 LINE 4 — DETAILED BREAKDOWN OF EXPENSES ON BOOKS NOT DEDUCTED ON RETURN</t>
         </is>
@@ -9376,6 +9510,7 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
     <row r="39" ht="21.75" customHeight="1" s="104">
       <c r="A39" s="108" t="inlineStr">
         <is>
@@ -9491,6 +9626,7 @@
         <v/>
       </c>
     </row>
+    <row r="49"/>
     <row r="50" ht="15" customHeight="1" s="104">
       <c r="A50" s="109" t="n"/>
       <c r="B50" s="110" t="n"/>
@@ -9601,7 +9737,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="104">
-      <c r="A1" s="105" t="inlineStr">
+      <c r="A1" s="217" t="inlineStr">
         <is>
           <t>SCHEDULE M-2 — PARTNERS' CAPITAL ACCOUNT RECONCILIATION WORKPAPER</t>
         </is>
@@ -9614,6 +9750,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="104">
       <c r="A4" s="107" t="inlineStr">
         <is>
@@ -9652,7 +9789,7 @@
       </c>
     </row>
     <row r="5" ht="21.75" customHeight="1" s="104">
-      <c r="A5" s="108" t="inlineStr">
+      <c r="A5" s="211" t="inlineStr">
         <is>
           <t>M-2 CAPITAL ACCOUNT RECONCILIATION</t>
         </is>
@@ -9953,6 +10090,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="21.75" customHeight="1" s="104">
       <c r="A16" s="143" t="n"/>
       <c r="B16" s="144" t="inlineStr">
@@ -9977,6 +10115,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="21.75" customHeight="1" s="104">
       <c r="A18" s="108" t="inlineStr">
         <is>
@@ -10226,7 +10365,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="104">
-      <c r="A1" s="105" t="inlineStr">
+      <c r="A1" s="217" t="inlineStr">
         <is>
           <t>SCHEDULE M-3 (FORM 1065) — NET INCOME RECONCILIATION WORKPAPER</t>
         </is>
@@ -10246,6 +10385,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="21.75" customHeight="1" s="104">
       <c r="A5" s="108" t="inlineStr">
         <is>
@@ -10601,6 +10741,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" ht="21.75" customHeight="1" s="104">
       <c r="A19" s="108" t="inlineStr">
         <is>
@@ -10875,6 +11016,7 @@
       <c r="H26" s="153" t="n"/>
       <c r="I26" s="145" t="n"/>
     </row>
+    <row r="27"/>
     <row r="28" ht="21.75" customHeight="1" s="104">
       <c r="A28" s="108" t="inlineStr">
         <is>
@@ -11761,7 +11903,7 @@
     </row>
     <row r="53" ht="21.75" customHeight="1" s="104"/>
     <row r="54" ht="15" customHeight="1" s="104">
-      <c r="A54" s="108" t="inlineStr">
+      <c r="A54" s="218" t="inlineStr">
         <is>
           <t>RECONCILIATION TOTALS AND TIE-OUTS</t>
         </is>
@@ -12134,6 +12276,7 @@
         <v/>
       </c>
     </row>
+    <row r="76"/>
     <row r="77" ht="15" customHeight="1" s="104">
       <c r="B77" s="161" t="inlineStr">
         <is>
@@ -12319,6 +12462,7 @@
         <v/>
       </c>
     </row>
+    <row r="91"/>
     <row r="92" ht="15" customHeight="1" s="104">
       <c r="C92" s="140" t="inlineStr">
         <is>
@@ -12363,7 +12507,7 @@
       <c r="A95" s="103" t="n"/>
     </row>
     <row r="96" ht="429" customHeight="1" s="104">
-      <c r="A96" s="162" t="inlineStr">
+      <c r="A96" s="219" t="inlineStr">
         <is>
           <t>NOTE: Schedule M-3 required if: (a) total assets &gt;= $10M, (b) 250+ K-1s, or (c) voluntary election. This workpaper serves as a detailed book-to-tax bridge in M-3 format for any client. Hide rows for items that don't apply.</t>
         </is>
@@ -12426,6 +12570,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="104">
       <c r="A5" s="166" t="inlineStr">
         <is>
@@ -12440,6 +12585,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8" ht="15" customHeight="1" s="104">
       <c r="A8" s="167" t="inlineStr">
         <is>
@@ -12503,7 +12649,7 @@
       </c>
     </row>
     <row r="9" ht="21.75" customHeight="1" s="104">
-      <c r="A9" s="168" t="inlineStr">
+      <c r="A9" s="220" t="inlineStr">
         <is>
           <t>INCOME ADJUSTMENTS</t>
         </is>
@@ -13988,8 +14134,9 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
     <row r="39" ht="15" customHeight="1" s="104">
-      <c r="A39" s="180" t="inlineStr">
+      <c r="A39" s="221" t="inlineStr">
         <is>
           <t>CHECKLIST TOTALS</t>
         </is>
@@ -13998,15 +14145,15 @@
       <c r="C39" s="169" t="n"/>
       <c r="D39" s="169" t="n"/>
       <c r="E39" s="170" t="n"/>
-      <c r="F39" s="181">
+      <c r="F39" s="222">
         <f>SUM(F9:F37)</f>
         <v/>
       </c>
-      <c r="G39" s="182">
+      <c r="G39" s="223">
         <f>SUM(G9:G37)</f>
         <v/>
       </c>
-      <c r="H39" s="181">
+      <c r="H39" s="222">
         <f>SUM(H9:H37)</f>
         <v/>
       </c>
@@ -14016,16 +14163,18 @@
       <c r="L39" s="112" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1" s="104">
-      <c r="A40" s="183" t="inlineStr">
+      <c r="A40" s="224" t="inlineStr">
         <is>
           <t>CHECK: Net Adjustment (Tax Total - Book Total) should match sum of Adj column</t>
         </is>
       </c>
-      <c r="G40" s="184">
+      <c r="G40" s="222">
         <f>H39-F39-G39</f>
         <v/>
       </c>
     </row>
+    <row r="41"/>
+    <row r="42"/>
     <row r="43" ht="24" customHeight="1" s="104">
       <c r="A43" s="166" t="inlineStr">
         <is>
@@ -14040,6 +14189,7 @@
         </is>
       </c>
     </row>
+    <row r="45"/>
     <row r="46" ht="15" customHeight="1" s="104">
       <c r="A46" s="167" t="inlineStr">
         <is>
@@ -15811,8 +15961,9 @@
       <c r="I96" s="112" t="n"/>
       <c r="J96" s="112" t="n"/>
     </row>
+    <row r="97"/>
     <row r="98" ht="15" customHeight="1" s="104">
-      <c r="A98" s="180" t="inlineStr">
+      <c r="A98" s="221" t="inlineStr">
         <is>
           <t>AJE TOTALS</t>
         </is>
@@ -15820,15 +15971,15 @@
       <c r="B98" s="169" t="n"/>
       <c r="C98" s="169" t="n"/>
       <c r="D98" s="170" t="n"/>
-      <c r="E98" s="181">
+      <c r="E98" s="222">
         <f>SUM(E47:E96)</f>
         <v/>
       </c>
-      <c r="F98" s="181">
+      <c r="F98" s="222">
         <f>SUM(F47:F96)</f>
         <v/>
       </c>
-      <c r="G98" s="181">
+      <c r="G98" s="222">
         <f>E98-F98</f>
         <v/>
       </c>
@@ -15837,16 +15988,18 @@
       <c r="J98" s="112" t="n"/>
     </row>
     <row r="99" ht="15" customHeight="1" s="104">
-      <c r="A99" s="183" t="inlineStr">
+      <c r="A99" s="224" t="inlineStr">
         <is>
           <t>CHECK: DR Total = CR Total (should be ZERO)</t>
         </is>
       </c>
-      <c r="G99" s="184">
+      <c r="G99" s="222">
         <f>E98-F98</f>
         <v/>
       </c>
     </row>
+    <row r="100"/>
+    <row r="101"/>
     <row r="102" ht="24" customHeight="1" s="104">
       <c r="A102" s="166" t="inlineStr">
         <is>
@@ -15854,6 +16007,7 @@
         </is>
       </c>
     </row>
+    <row r="103"/>
     <row r="104" ht="15" customHeight="1" s="104">
       <c r="A104" s="167" t="inlineStr">
         <is>
@@ -15887,7 +16041,7 @@
       </c>
     </row>
     <row r="105" ht="21.75" customHeight="1" s="104">
-      <c r="A105" s="172" t="inlineStr">
+      <c r="A105" s="225" t="inlineStr">
         <is>
           <t>Page 1 — Income (L8)</t>
         </is>
@@ -15915,7 +16069,7 @@
       </c>
     </row>
     <row r="106" ht="21.75" customHeight="1" s="104">
-      <c r="A106" s="172" t="inlineStr">
+      <c r="A106" s="225" t="inlineStr">
         <is>
           <t>Page 1 — Deductions (L21)</t>
         </is>
@@ -15943,7 +16097,7 @@
       </c>
     </row>
     <row r="107" ht="21.75" customHeight="1" s="104">
-      <c r="A107" s="172" t="inlineStr">
+      <c r="A107" s="225" t="inlineStr">
         <is>
           <t>Page 1 — OBI (L22)</t>
         </is>
@@ -15971,63 +16125,63 @@
       </c>
     </row>
     <row r="108" ht="21.75" customHeight="1" s="104">
-      <c r="A108" s="172" t="inlineStr">
+      <c r="A108" s="226" t="inlineStr">
         <is>
           <t>Schedule K — Total</t>
         </is>
       </c>
-      <c r="B108" s="175">
+      <c r="B108" s="227">
         <f>'Working Trial Balance'!D82</f>
         <v/>
       </c>
-      <c r="C108" s="189">
+      <c r="C108" s="228">
         <f>'Working Trial Balance'!H82-'Working Trial Balance'!D82</f>
         <v/>
       </c>
-      <c r="D108" s="175">
+      <c r="D108" s="227">
         <f>'Working Trial Balance'!H82</f>
         <v/>
       </c>
-      <c r="E108" s="174" t="inlineStr">
+      <c r="E108" s="229" t="inlineStr">
         <is>
           <t>WTB R82</t>
         </is>
       </c>
-      <c r="F108" s="190">
+      <c r="F108" s="230">
         <f>IF(D108=B108+C108,"✓","✗")</f>
         <v/>
       </c>
     </row>
     <row r="109" ht="21.75" customHeight="1" s="104">
-      <c r="A109" s="172" t="inlineStr">
+      <c r="A109" s="226" t="inlineStr">
         <is>
           <t>Schedule L — Total Assets</t>
         </is>
       </c>
-      <c r="B109" s="175">
+      <c r="B109" s="227">
         <f>'Working Trial Balance'!D12</f>
         <v/>
       </c>
-      <c r="C109" s="189">
+      <c r="C109" s="228">
         <f>'Working Trial Balance'!H12-'Working Trial Balance'!D12</f>
         <v/>
       </c>
-      <c r="D109" s="175">
+      <c r="D109" s="227">
         <f>'Working Trial Balance'!H12</f>
         <v/>
       </c>
-      <c r="E109" s="174" t="inlineStr">
+      <c r="E109" s="229" t="inlineStr">
         <is>
           <t>WTB R12</t>
         </is>
       </c>
-      <c r="F109" s="190">
+      <c r="F109" s="230">
         <f>IF(D109=B109+C109,"✓","✗")</f>
         <v/>
       </c>
     </row>
     <row r="110" ht="21.75" customHeight="1" s="104">
-      <c r="A110" s="172" t="inlineStr">
+      <c r="A110" s="225" t="inlineStr">
         <is>
           <t>Schedule L — Liabilities</t>
         </is>
@@ -16055,7 +16209,7 @@
       </c>
     </row>
     <row r="111" ht="21.75" customHeight="1" s="104">
-      <c r="A111" s="172" t="inlineStr">
+      <c r="A111" s="225" t="inlineStr">
         <is>
           <t>M-2 — Ending Capital</t>
         </is>
@@ -16083,7 +16237,7 @@
       </c>
     </row>
     <row r="112" ht="21.75" customHeight="1" s="104">
-      <c r="A112" s="172" t="inlineStr">
+      <c r="A112" s="226" t="inlineStr">
         <is>
           <t>M-1 Line 9 = K Total</t>
         </is>
@@ -16091,16 +16245,18 @@
       <c r="B112" s="191" t="n"/>
       <c r="C112" s="192" t="n"/>
       <c r="D112" s="191" t="n"/>
-      <c r="E112" s="174" t="inlineStr">
+      <c r="E112" s="229" t="inlineStr">
         <is>
           <t>WTB R103</t>
         </is>
       </c>
-      <c r="F112" s="190">
+      <c r="F112" s="230">
         <f>IF('Working Trial Balance'!H103=0,"✓","✗")</f>
         <v/>
       </c>
     </row>
+    <row r="113"/>
+    <row r="114"/>
     <row r="115" ht="24" customHeight="1" s="104">
       <c r="A115" s="166" t="inlineStr">
         <is>
@@ -16108,6 +16264,7 @@
         </is>
       </c>
     </row>
+    <row r="116"/>
     <row r="117" ht="15" customHeight="1" s="104">
       <c r="A117" s="167" t="inlineStr">
         <is>
@@ -16647,6 +16804,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="25.5" customHeight="1" s="104">
       <c r="A5" s="166" t="inlineStr">
         <is>
@@ -16654,6 +16812,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="21.75" customHeight="1" s="104">
       <c r="A7" s="195" t="inlineStr">
         <is>
@@ -16796,6 +16955,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="21.75" customHeight="1" s="104">
       <c r="A14" s="168" t="inlineStr">
         <is>
@@ -16961,6 +17121,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" ht="21.75" customHeight="1" s="104">
       <c r="A19" s="168" t="inlineStr">
         <is>
@@ -17203,6 +17364,7 @@
       </c>
       <c r="K28" s="112" t="n"/>
     </row>
+    <row r="29"/>
     <row r="30" ht="25.5" customHeight="1" s="104">
       <c r="A30" s="166" t="inlineStr">
         <is>
@@ -17210,6 +17372,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32" ht="21.75" customHeight="1" s="104">
       <c r="A32" s="195" t="inlineStr">
         <is>
@@ -17372,6 +17535,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40" ht="21.75" customHeight="1" s="104">
       <c r="A40" s="168" t="inlineStr">
         <is>
@@ -17603,6 +17767,7 @@
         </is>
       </c>
     </row>
+    <row r="45"/>
     <row r="46" ht="21.75" customHeight="1" s="104">
       <c r="A46" s="168" t="inlineStr">
         <is>
@@ -17870,6 +18035,7 @@
       </c>
       <c r="K56" s="112" t="n"/>
     </row>
+    <row r="57"/>
     <row r="58" ht="25.5" customHeight="1" s="104">
       <c r="A58" s="166" t="inlineStr">
         <is>
@@ -17877,6 +18043,7 @@
         </is>
       </c>
     </row>
+    <row r="59"/>
     <row r="60" ht="21.75" customHeight="1" s="104">
       <c r="A60" s="195" t="inlineStr">
         <is>
@@ -18015,6 +18182,7 @@
         </is>
       </c>
     </row>
+    <row r="66"/>
     <row r="67" ht="21.75" customHeight="1" s="104">
       <c r="A67" s="168" t="inlineStr">
         <is>
@@ -18074,6 +18242,7 @@
       <c r="J69" s="169" t="n"/>
       <c r="K69" s="169" t="n"/>
     </row>
+    <row r="70"/>
     <row r="71" ht="15" customHeight="1" s="104">
       <c r="A71" s="167" t="inlineStr">
         <is>
@@ -18237,6 +18406,7 @@
         </is>
       </c>
     </row>
+    <row r="74"/>
     <row r="75" ht="21.75" customHeight="1" s="104">
       <c r="A75" s="168" t="inlineStr">
         <is>
@@ -18479,6 +18649,7 @@
       </c>
       <c r="K84" s="112" t="n"/>
     </row>
+    <row r="85"/>
     <row r="86" ht="25.5" customHeight="1" s="104">
       <c r="A86" s="166" t="inlineStr">
         <is>
@@ -18486,6 +18657,7 @@
         </is>
       </c>
     </row>
+    <row r="87"/>
     <row r="88" ht="21.75" customHeight="1" s="104">
       <c r="A88" s="195" t="inlineStr">
         <is>
@@ -18648,6 +18820,7 @@
         </is>
       </c>
     </row>
+    <row r="95"/>
     <row r="96" ht="21.75" customHeight="1" s="104">
       <c r="A96" s="168" t="inlineStr">
         <is>
@@ -18874,6 +19047,7 @@
         </is>
       </c>
     </row>
+    <row r="101"/>
     <row r="102" ht="21.75" customHeight="1" s="104">
       <c r="A102" s="168" t="inlineStr">
         <is>
@@ -19041,6 +19215,7 @@
       </c>
       <c r="K108" s="112" t="n"/>
     </row>
+    <row r="109"/>
     <row r="110" ht="25.5" customHeight="1" s="104">
       <c r="A110" s="166" t="inlineStr">
         <is>
@@ -19048,6 +19223,7 @@
         </is>
       </c>
     </row>
+    <row r="111"/>
     <row r="112" ht="21.75" customHeight="1" s="104">
       <c r="A112" s="195" t="inlineStr">
         <is>
@@ -19258,6 +19434,7 @@
         </is>
       </c>
     </row>
+    <row r="121"/>
     <row r="122" ht="21.75" customHeight="1" s="104">
       <c r="A122" s="168" t="inlineStr">
         <is>
@@ -19497,6 +19674,7 @@
         </is>
       </c>
     </row>
+    <row r="128"/>
     <row r="129" ht="21.75" customHeight="1" s="104">
       <c r="A129" s="168" t="inlineStr">
         <is>
@@ -19739,6 +19917,7 @@
       </c>
       <c r="K138" s="112" t="n"/>
     </row>
+    <row r="139"/>
     <row r="140" ht="25.5" customHeight="1" s="104">
       <c r="A140" s="166" t="inlineStr">
         <is>
@@ -19746,6 +19925,7 @@
         </is>
       </c>
     </row>
+    <row r="141"/>
     <row r="142" ht="21.75" customHeight="1" s="104">
       <c r="A142" s="195" t="inlineStr">
         <is>
@@ -19884,6 +20064,7 @@
         </is>
       </c>
     </row>
+    <row r="148"/>
     <row r="149" ht="21.75" customHeight="1" s="104">
       <c r="A149" s="168" t="inlineStr">
         <is>
@@ -20032,6 +20213,7 @@
         </is>
       </c>
     </row>
+    <row r="153"/>
     <row r="154" ht="21.75" customHeight="1" s="104">
       <c r="A154" s="168" t="inlineStr">
         <is>
@@ -20224,6 +20406,7 @@
       </c>
       <c r="K161" s="112" t="n"/>
     </row>
+    <row r="162"/>
     <row r="163" ht="25.5" customHeight="1" s="104">
       <c r="A163" s="166" t="inlineStr">
         <is>
@@ -20231,6 +20414,7 @@
         </is>
       </c>
     </row>
+    <row r="164"/>
     <row r="165" ht="21.75" customHeight="1" s="104">
       <c r="A165" s="195" t="inlineStr">
         <is>
@@ -20369,6 +20553,7 @@
         </is>
       </c>
     </row>
+    <row r="171"/>
     <row r="172" ht="21.75" customHeight="1" s="104">
       <c r="A172" s="168" t="inlineStr">
         <is>
@@ -20568,6 +20753,7 @@
         </is>
       </c>
     </row>
+    <row r="177"/>
     <row r="178" ht="21.75" customHeight="1" s="104">
       <c r="A178" s="168" t="inlineStr">
         <is>
@@ -20735,6 +20921,7 @@
       </c>
       <c r="K184" s="112" t="n"/>
     </row>
+    <row r="185"/>
     <row r="186" ht="25.5" customHeight="1" s="104">
       <c r="A186" s="166" t="inlineStr">
         <is>
@@ -20742,6 +20929,7 @@
         </is>
       </c>
     </row>
+    <row r="187"/>
     <row r="188" ht="21.75" customHeight="1" s="104">
       <c r="A188" s="195" t="inlineStr">
         <is>
@@ -20880,6 +21068,7 @@
         </is>
       </c>
     </row>
+    <row r="194"/>
     <row r="195" ht="21.75" customHeight="1" s="104">
       <c r="A195" s="168" t="inlineStr">
         <is>
@@ -21044,6 +21233,7 @@
         </is>
       </c>
     </row>
+    <row r="199"/>
     <row r="200" ht="21.75" customHeight="1" s="104">
       <c r="A200" s="168" t="inlineStr">
         <is>
@@ -21161,6 +21351,8 @@
       </c>
       <c r="K204" s="112" t="n"/>
     </row>
+    <row r="205"/>
+    <row r="206"/>
     <row r="207" ht="25.5" customHeight="1" s="104">
       <c r="A207" s="166" t="inlineStr">
         <is>
@@ -21168,6 +21360,7 @@
         </is>
       </c>
     </row>
+    <row r="208"/>
     <row r="209" ht="15" customHeight="1" s="104">
       <c r="A209" s="167" t="inlineStr">
         <is>
@@ -21739,6 +21932,8 @@
         </is>
       </c>
     </row>
+    <row r="218"/>
+    <row r="219"/>
     <row r="220" ht="21.75" customHeight="1" s="104">
       <c r="A220" s="205" t="inlineStr">
         <is>

</xml_diff>